<commit_message>
Nueva reserva Minha Kim (HMZJ8DHXZA, abr 2027) + notas 31/08 pendientes de comitear
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P1UqJsY48mdHjF1TsSD7kc
</commit_message>
<xml_diff>
--- a/output/pricing_output.xlsx
+++ b/output/pricing_output.xlsx
@@ -461,7 +461,7 @@
     <col width="14" customWidth="1" min="19" max="19"/>
     <col width="14" customWidth="1" min="20" max="20"/>
     <col width="13" customWidth="1" min="21" max="21"/>
-    <col width="43" customWidth="1" min="22" max="22"/>
+    <col width="46" customWidth="1" min="22" max="22"/>
     <col width="13" customWidth="1" min="23" max="23"/>
     <col width="17" customWidth="1" min="24" max="24"/>
   </cols>
@@ -613,7 +613,7 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="G2" s="2" t="n">
         <v>42.2</v>
@@ -646,22 +646,18 @@
         </is>
       </c>
       <c r="O2" s="2" t="n">
-        <v>62.66</v>
+        <v>62.42</v>
       </c>
       <c r="P2" s="2" t="n">
-        <v>56.39</v>
+        <v>56.18</v>
       </c>
       <c r="Q2" s="2" t="n"/>
       <c r="R2" s="2" t="inlineStr">
         <is>
-          <t>Equilibrio (temporada media + antelación adecuada). Precio de mercado balanceado. Ajustes en zona: pickup fuerte (↑10%) + hueco muy corto (↓10%).</t>
-        </is>
-      </c>
-      <c r="S2" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-02</t>
-        </is>
-      </c>
+          <t>Equilibrio (temporada media). Precio de mercado balanceado. Ajustes en zona: pickup fuerte (↑10%) + hueco muy corto (↓10%).</t>
+        </is>
+      </c>
+      <c r="S2" s="2" t="n"/>
       <c r="T2" s="2" t="inlineStr">
         <is>
           <t>2026-09-17</t>
@@ -674,7 +670,7 @@
       </c>
       <c r="V2" s="2" t="inlineStr">
         <is>
-          <t>Revisar 2026-09-02; sin vender → bajar 5%</t>
+          <t>Revisar 2026-09-17; sin vender → bajar 5–10%</t>
         </is>
       </c>
       <c r="W2" s="2" t="n">
@@ -709,7 +705,7 @@
         </is>
       </c>
       <c r="F3" s="3" t="n">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="G3" s="3" t="n">
         <v>33.3</v>
@@ -805,7 +801,7 @@
         </is>
       </c>
       <c r="F4" s="3" t="n">
-        <v>49</v>
+        <v>41</v>
       </c>
       <c r="G4" s="3" t="n">
         <v>26.7</v>
@@ -901,7 +897,7 @@
         </is>
       </c>
       <c r="F5" s="3" t="n">
-        <v>54</v>
+        <v>46</v>
       </c>
       <c r="G5" s="3" t="n">
         <v>22.2</v>
@@ -997,7 +993,7 @@
         </is>
       </c>
       <c r="F6" s="2" t="n">
-        <v>62</v>
+        <v>54</v>
       </c>
       <c r="G6" s="2" t="n">
         <v>15.6</v>
@@ -1026,21 +1022,21 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>buena antelación (↑15%) + pickup fuerte (↑10%) + baja ocupación futura (↓10%)</t>
+          <t>pickup fuerte (↑10%) + baja ocupación futura (↓10%)</t>
         </is>
       </c>
       <c r="O6" s="2" t="n">
-        <v>48.4</v>
+        <v>48.3</v>
       </c>
       <c r="P6" s="2" t="n">
-        <v>43.56</v>
+        <v>43.47</v>
       </c>
       <c r="Q6" s="2" t="n">
-        <v>321.86</v>
+        <v>321.19</v>
       </c>
       <c r="R6" s="2" t="inlineStr">
         <is>
-          <t>Equilibrio (temporada baja + antelación adecuada). Precio de mercado balanceado. Ajustes en zona: buena antelación (↑15%) + pickup fuerte (↑10%) + baja ocupación futura (↓10%).</t>
+          <t>Equilibrio (temporada baja + antelación adecuada). Precio de mercado balanceado. Ajustes en zona: pickup fuerte (↑10%) + baja ocupación futura (↓10%).</t>
         </is>
       </c>
       <c r="S6" s="2" t="inlineStr">
@@ -1095,7 +1091,7 @@
         </is>
       </c>
       <c r="F7" s="2" t="n">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="G7" s="2" t="n">
         <v>11.1</v>
@@ -1771,7 +1767,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-08</t>
         </is>
       </c>
     </row>
@@ -1807,7 +1803,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>1.044 (auto — vs 1.044 auto)</t>
+          <t>1.025 (auto — vs 1.025 auto)</t>
         </is>
       </c>
     </row>
@@ -1819,7 +1815,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>1.044</t>
+          <t>1.025</t>
         </is>
       </c>
     </row>
@@ -2036,12 +2032,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-08-31 12:48:53</t>
+          <t>2026-09-08 15:10:12</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -2056,12 +2052,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.044</t>
+          <t>1.025</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>1.044</t>
+          <t>1.025</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">

</xml_diff>

<commit_message>
Backlog 21/09 (visitas ago, 2 reviews, 5 reservas, cancelacion Minha Kim) + 2 reservas nuevas (Llorens Coll, Monika Schindler)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/pricing_output.xlsx
+++ b/output/pricing_output.xlsx
@@ -46,12 +46,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
+        <fgColor rgb="00FDE9D9"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FDE9D9"/>
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -461,7 +461,7 @@
     <col width="14" customWidth="1" min="19" max="19"/>
     <col width="14" customWidth="1" min="20" max="20"/>
     <col width="13" customWidth="1" min="21" max="21"/>
-    <col width="46" customWidth="1" min="22" max="22"/>
+    <col width="51" customWidth="1" min="22" max="22"/>
     <col width="13" customWidth="1" min="23" max="23"/>
     <col width="17" customWidth="1" min="24" max="24"/>
   </cols>
@@ -591,16 +591,16 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
@@ -613,554 +613,542 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>42.2</v>
+        <v>41.1</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>52.25</v>
+        <v>52.33</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>60.27</v>
+        <v>60.33</v>
       </c>
       <c r="J2" s="2" t="n">
-        <v>67.25</v>
+        <v>68</v>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>Equilibrio</t>
+          <t>Ocupación</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>P45–P60  (60€–65€)</t>
+          <t>P25–P40  (52€–57€)</t>
         </is>
       </c>
       <c r="M2" s="2" t="n">
-        <v>62.42</v>
+        <v>54.56</v>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>pickup fuerte (↑10%) + hueco muy corto (↓10%)</t>
+          <t>baja antelación (↓10%) + pickup fuerte (↑10%) + hueco muy corto (↓10%)</t>
         </is>
       </c>
       <c r="O2" s="2" t="n">
-        <v>62.42</v>
+        <v>54.12</v>
       </c>
       <c r="P2" s="2" t="n">
-        <v>56.18</v>
+        <v>48.71</v>
       </c>
       <c r="Q2" s="2" t="n"/>
       <c r="R2" s="2" t="inlineStr">
         <is>
-          <t>Equilibrio (temporada media). Precio de mercado balanceado. Ajustes en zona: pickup fuerte (↑10%) + hueco muy corto (↓10%).</t>
+          <t>Ocupación (hueco muy corto + baja antelación). Objetivo: convertir rápido, evitar hueco vacío. Ajustes en zona: baja antelación (↓10%) + pickup fuerte (↑10%) + hueco muy corto (↓10%).</t>
         </is>
       </c>
       <c r="S2" s="2" t="n"/>
-      <c r="T2" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-17</t>
-        </is>
-      </c>
+      <c r="T2" s="2" t="n"/>
       <c r="U2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="V2" s="2" t="inlineStr">
         <is>
-          <t>Revisar 2026-09-17; sin vender → bajar 5–10%</t>
+          <t>Revisar 2026-10-05; sin vender → precio Ocupación</t>
         </is>
       </c>
       <c r="W2" s="2" t="n">
-        <v>52.25</v>
+        <v>47.1</v>
       </c>
       <c r="X2" s="2" t="n">
-        <v>75.98999999999999</v>
+        <v>76.84</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Octubre</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>media</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>34.4</v>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>52.33</v>
+      </c>
+      <c r="I3" s="2" t="n">
+        <v>60.33</v>
+      </c>
+      <c r="J3" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>Ocupación</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>P25–P40  (52€–57€)</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="n">
+        <v>54.56</v>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>pickup fuerte (↑10%) + hueco muy corto (↓10%)</t>
+        </is>
+      </c>
+      <c r="O3" s="2" t="n">
+        <v>54.56</v>
+      </c>
+      <c r="P3" s="2" t="n">
+        <v>49.1</v>
+      </c>
+      <c r="Q3" s="2" t="n"/>
+      <c r="R3" s="2" t="inlineStr">
+        <is>
+          <t>Ocupación (hueco muy corto + baja ocupación futura). Objetivo: convertir rápido, evitar hueco vacío. Ajustes en zona: pickup fuerte (↑10%) + hueco muy corto (↓10%).</t>
+        </is>
+      </c>
+      <c r="S3" s="2" t="n"/>
+      <c r="T3" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="U3" s="2" t="inlineStr">
         <is>
           <t>2026-10-12</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-13</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="V3" s="2" t="inlineStr">
+        <is>
+          <t>Revisar 2026-10-04; sin vender → bajar 5–10%</t>
+        </is>
+      </c>
+      <c r="W3" s="2" t="n">
+        <v>47.1</v>
+      </c>
+      <c r="X3" s="2" t="n">
+        <v>76.84</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>Octubre</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>media</t>
         </is>
       </c>
-      <c r="F3" s="3" t="n">
-        <v>34</v>
-      </c>
-      <c r="G3" s="3" t="n">
-        <v>33.3</v>
-      </c>
-      <c r="H3" s="3" t="n">
-        <v>52.25</v>
-      </c>
-      <c r="I3" s="3" t="n">
-        <v>60.27</v>
-      </c>
-      <c r="J3" s="3" t="n">
-        <v>67.25</v>
-      </c>
-      <c r="K3" s="3" t="inlineStr">
+      <c r="F4" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>52.33</v>
+      </c>
+      <c r="I4" s="2" t="n">
+        <v>60.33</v>
+      </c>
+      <c r="J4" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>Ocupación</t>
         </is>
       </c>
-      <c r="L3" s="3" t="inlineStr">
-        <is>
-          <t>P25–P40  (52€–56€)</t>
-        </is>
-      </c>
-      <c r="M3" s="3" t="n">
-        <v>54.1</v>
-      </c>
-      <c r="N3" s="3" t="inlineStr">
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>P25–P40  (52€–57€)</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="n">
+        <v>54.56</v>
+      </c>
+      <c r="N4" s="2" t="inlineStr">
         <is>
           <t>pickup fuerte (↑10%) + hueco muy corto (↓10%)</t>
         </is>
       </c>
-      <c r="O3" s="3" t="n">
-        <v>54.28</v>
-      </c>
-      <c r="P3" s="3" t="n">
-        <v>48.85</v>
-      </c>
-      <c r="Q3" s="3" t="n"/>
-      <c r="R3" s="3" t="inlineStr">
+      <c r="O4" s="2" t="n">
+        <v>54.56</v>
+      </c>
+      <c r="P4" s="2" t="n">
+        <v>49.1</v>
+      </c>
+      <c r="Q4" s="2" t="n"/>
+      <c r="R4" s="2" t="inlineStr">
         <is>
           <t>Ocupación (hueco muy corto + baja ocupación futura). Objetivo: convertir rápido, evitar hueco vacío. Ajustes en zona: pickup fuerte (↑10%) + hueco muy corto (↓10%).</t>
         </is>
       </c>
-      <c r="S3" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-12</t>
-        </is>
-      </c>
-      <c r="T3" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-27</t>
-        </is>
-      </c>
-      <c r="U3" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-05</t>
-        </is>
-      </c>
-      <c r="V3" s="3" t="inlineStr">
-        <is>
-          <t>Revisar 2026-09-12; sin vender → bajar 5%</t>
-        </is>
-      </c>
-      <c r="W3" s="3" t="n">
-        <v>47.02</v>
-      </c>
-      <c r="X3" s="3" t="n">
-        <v>75.98999999999999</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>Octubre</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>media</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="n">
-        <v>41</v>
-      </c>
-      <c r="G4" s="3" t="n">
-        <v>26.7</v>
-      </c>
-      <c r="H4" s="3" t="n">
-        <v>52.25</v>
-      </c>
-      <c r="I4" s="3" t="n">
-        <v>60.27</v>
-      </c>
-      <c r="J4" s="3" t="n">
-        <v>67.25</v>
-      </c>
-      <c r="K4" s="3" t="inlineStr">
-        <is>
-          <t>Ocupación</t>
-        </is>
-      </c>
-      <c r="L4" s="3" t="inlineStr">
-        <is>
-          <t>P25–P40  (52€–56€)</t>
-        </is>
-      </c>
-      <c r="M4" s="3" t="n">
-        <v>54.1</v>
-      </c>
-      <c r="N4" s="3" t="inlineStr">
-        <is>
-          <t>pickup fuerte (↑10%) + hueco muy corto (↓10%) + baja ocupación futura (↓10%)</t>
-        </is>
-      </c>
-      <c r="O4" s="3" t="n">
-        <v>53.91</v>
-      </c>
-      <c r="P4" s="3" t="n">
-        <v>48.52</v>
-      </c>
-      <c r="Q4" s="3" t="n"/>
-      <c r="R4" s="3" t="inlineStr">
-        <is>
-          <t>Ocupación (hueco muy corto + baja ocupación futura). Objetivo: convertir rápido, evitar hueco vacío. Ajustes en zona: pickup fuerte (↑10%) + hueco muy corto (↓10%) + baja ocupación futura (↓10%).</t>
-        </is>
-      </c>
-      <c r="S4" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-      <c r="T4" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-04</t>
-        </is>
-      </c>
-      <c r="U4" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-12</t>
-        </is>
-      </c>
-      <c r="V4" s="3" t="inlineStr">
-        <is>
-          <t>Revisar 2026-09-19; sin vender → bajar 5%</t>
-        </is>
-      </c>
-      <c r="W4" s="3" t="n">
-        <v>47.02</v>
-      </c>
-      <c r="X4" s="3" t="n">
-        <v>75.98999999999999</v>
+      <c r="S4" s="2" t="n"/>
+      <c r="T4" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="U4" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="V4" s="2" t="inlineStr">
+        <is>
+          <t>Revisar 2026-10-09; sin vender → bajar 5–10%</t>
+        </is>
+      </c>
+      <c r="W4" s="2" t="n">
+        <v>52.33</v>
+      </c>
+      <c r="X4" s="2" t="n">
+        <v>76.84</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-11-01</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-11-07</t>
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Octubre</t>
+          <t>Noviembre</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>media</t>
+          <t>baja</t>
         </is>
       </c>
       <c r="F5" s="3" t="n">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>22.2</v>
+        <v>23.3</v>
       </c>
       <c r="H5" s="3" t="n">
-        <v>52.25</v>
+        <v>44.01</v>
       </c>
       <c r="I5" s="3" t="n">
-        <v>60.27</v>
+        <v>47.75</v>
       </c>
       <c r="J5" s="3" t="n">
-        <v>67.25</v>
+        <v>50</v>
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>Ocupación</t>
+          <t>Equilibrio</t>
         </is>
       </c>
       <c r="L5" s="3" t="inlineStr">
         <is>
-          <t>P25–P40  (52€–56€)</t>
+          <t>P45–P60  (48€–49€)</t>
         </is>
       </c>
       <c r="M5" s="3" t="n">
-        <v>54.1</v>
+        <v>48.46</v>
       </c>
       <c r="N5" s="3" t="inlineStr">
         <is>
-          <t>pickup fuerte (↑10%) + hueco muy corto (↓10%) + baja ocupación futura (↓10%)</t>
+          <t>pickup fuerte (↑10%) + baja ocupación futura (↓10%)</t>
         </is>
       </c>
       <c r="O5" s="3" t="n">
-        <v>53.91</v>
+        <v>48.53</v>
       </c>
       <c r="P5" s="3" t="n">
-        <v>48.52</v>
+        <v>43.68</v>
       </c>
       <c r="Q5" s="3" t="n"/>
       <c r="R5" s="3" t="inlineStr">
         <is>
-          <t>Ocupación (hueco muy corto + baja ocupación futura). Objetivo: convertir rápido, evitar hueco vacío. Ajustes en zona: pickup fuerte (↑10%) + hueco muy corto (↓10%) + baja ocupación futura (↓10%).</t>
+          <t>Equilibrio (temporada baja + antelación adecuada). Precio de mercado balanceado. Ajustes en zona: pickup fuerte (↑10%) + baja ocupación futura (↓10%).</t>
         </is>
       </c>
       <c r="S5" s="3" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="T5" s="3" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="U5" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="V5" s="3" t="inlineStr">
         <is>
-          <t>Revisar 2026-09-24; sin vender → bajar 5%</t>
+          <t>Revisar 2026-10-02; sin vender → bajar 5%</t>
         </is>
       </c>
       <c r="W5" s="3" t="n">
-        <v>52.25</v>
+        <v>44.01</v>
       </c>
       <c r="X5" s="3" t="n">
-        <v>75.98999999999999</v>
+        <v>56.5</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>2026-11-01</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>2026-11-14</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>2026-12-03</t>
         </is>
       </c>
-      <c r="C6" s="2" t="n">
-        <v>32</v>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="C6" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Noviembre</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="E6" s="3" t="inlineStr">
         <is>
           <t>baja</t>
         </is>
       </c>
-      <c r="F6" s="2" t="n">
-        <v>54</v>
-      </c>
-      <c r="G6" s="2" t="n">
-        <v>15.6</v>
-      </c>
-      <c r="H6" s="2" t="n">
-        <v>43.9</v>
-      </c>
-      <c r="I6" s="2" t="n">
+      <c r="F6" s="3" t="n">
+        <v>47</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>23.3</v>
+      </c>
+      <c r="H6" s="3" t="n">
+        <v>44.01</v>
+      </c>
+      <c r="I6" s="3" t="n">
         <v>47.75</v>
       </c>
-      <c r="J6" s="2" t="n">
+      <c r="J6" s="3" t="n">
         <v>50</v>
       </c>
-      <c r="K6" s="2" t="inlineStr">
+      <c r="K6" s="3" t="inlineStr">
         <is>
           <t>Equilibrio</t>
         </is>
       </c>
-      <c r="L6" s="2" t="inlineStr">
+      <c r="L6" s="3" t="inlineStr">
         <is>
           <t>P45–P60  (48€–49€)</t>
         </is>
       </c>
-      <c r="M6" s="2" t="n">
-        <v>48.17</v>
-      </c>
-      <c r="N6" s="2" t="inlineStr">
+      <c r="M6" s="3" t="n">
+        <v>48.46</v>
+      </c>
+      <c r="N6" s="3" t="inlineStr">
         <is>
           <t>pickup fuerte (↑10%) + baja ocupación futura (↓10%)</t>
         </is>
       </c>
-      <c r="O6" s="2" t="n">
-        <v>48.3</v>
-      </c>
-      <c r="P6" s="2" t="n">
-        <v>43.47</v>
-      </c>
-      <c r="Q6" s="2" t="n">
-        <v>321.19</v>
-      </c>
-      <c r="R6" s="2" t="inlineStr">
+      <c r="O6" s="3" t="n">
+        <v>48.53</v>
+      </c>
+      <c r="P6" s="3" t="n">
+        <v>43.68</v>
+      </c>
+      <c r="Q6" s="3" t="n">
+        <v>322.72</v>
+      </c>
+      <c r="R6" s="3" t="inlineStr">
         <is>
           <t>Equilibrio (temporada baja + antelación adecuada). Precio de mercado balanceado. Ajustes en zona: pickup fuerte (↑10%) + baja ocupación futura (↓10%).</t>
         </is>
       </c>
-      <c r="S6" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-02</t>
-        </is>
-      </c>
-      <c r="T6" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="U6" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-25</t>
-        </is>
-      </c>
-      <c r="V6" s="2" t="inlineStr">
-        <is>
-          <t>Revisar 2026-10-02; sin vender → bajar 5%</t>
-        </is>
-      </c>
-      <c r="W6" s="2" t="n">
-        <v>43.9</v>
-      </c>
-      <c r="X6" s="2" t="n">
+      <c r="S6" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="T6" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="U6" s="3" t="inlineStr">
+        <is>
+          <t>2026-11-07</t>
+        </is>
+      </c>
+      <c r="V6" s="3" t="inlineStr">
+        <is>
+          <t>Revisar 2026-10-15; sin vender → bajar 5%</t>
+        </is>
+      </c>
+      <c r="W6" s="3" t="n">
+        <v>44.01</v>
+      </c>
+      <c r="X6" s="3" t="n">
         <v>56.5</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>2026-12-07</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>2026-12-23</t>
         </is>
       </c>
-      <c r="C7" s="2" t="n">
+      <c r="C7" s="3" t="n">
         <v>16</v>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>Diciembre (1-19)</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="E7" s="3" t="inlineStr">
         <is>
           <t>baja</t>
         </is>
       </c>
-      <c r="F7" s="2" t="n">
-        <v>90</v>
-      </c>
-      <c r="G7" s="2" t="n">
-        <v>11.1</v>
-      </c>
-      <c r="H7" s="2" t="n">
+      <c r="F7" s="3" t="n">
+        <v>70</v>
+      </c>
+      <c r="G7" s="3" t="n">
+        <v>18.9</v>
+      </c>
+      <c r="H7" s="3" t="n">
         <v>42.03</v>
       </c>
-      <c r="I7" s="2" t="n">
+      <c r="I7" s="3" t="n">
         <v>43.45</v>
       </c>
-      <c r="J7" s="2" t="n">
+      <c r="J7" s="3" t="n">
         <v>46.67</v>
       </c>
-      <c r="K7" s="2" t="inlineStr">
+      <c r="K7" s="3" t="inlineStr">
         <is>
           <t>Equilibrio</t>
         </is>
       </c>
-      <c r="L7" s="2" t="inlineStr">
+      <c r="L7" s="3" t="inlineStr">
         <is>
           <t>P45–P60  (43€–45€)</t>
         </is>
       </c>
-      <c r="M7" s="2" t="n">
+      <c r="M7" s="3" t="n">
         <v>43.83</v>
       </c>
-      <c r="N7" s="2" t="inlineStr">
+      <c r="N7" s="3" t="inlineStr">
         <is>
           <t>buena antelación (↑15%) + pickup fuerte (↑10%) + baja ocupación futura (↓10%)</t>
         </is>
       </c>
-      <c r="O7" s="2" t="n">
+      <c r="O7" s="3" t="n">
         <v>44.07</v>
       </c>
-      <c r="P7" s="2" t="n">
+      <c r="P7" s="3" t="n">
         <v>39.66</v>
       </c>
-      <c r="Q7" s="2" t="n">
+      <c r="Q7" s="3" t="n">
         <v>293.07</v>
       </c>
-      <c r="R7" s="2" t="inlineStr">
+      <c r="R7" s="3" t="inlineStr">
         <is>
           <t>Equilibrio (temporada baja + antelación adecuada). Precio de mercado balanceado. Ajustes en zona: buena antelación (↑15%) + pickup fuerte (↑10%) + baja ocupación futura (↓10%).</t>
         </is>
       </c>
-      <c r="S7" s="2" t="inlineStr">
+      <c r="S7" s="3" t="inlineStr">
         <is>
           <t>2026-11-07</t>
         </is>
       </c>
-      <c r="T7" s="2" t="inlineStr">
+      <c r="T7" s="3" t="inlineStr">
         <is>
           <t>2026-11-22</t>
         </is>
       </c>
-      <c r="U7" s="2" t="inlineStr">
+      <c r="U7" s="3" t="inlineStr">
         <is>
           <t>2026-11-30</t>
         </is>
       </c>
-      <c r="V7" s="2" t="inlineStr">
+      <c r="V7" s="3" t="inlineStr">
         <is>
           <t>Revisar 2026-11-07; sin vender → bajar 5%</t>
         </is>
       </c>
-      <c r="W7" s="2" t="n">
+      <c r="W7" s="3" t="n">
         <v>42.03</v>
       </c>
-      <c r="X7" s="2" t="n">
+      <c r="X7" s="3" t="n">
         <v>52.74</v>
       </c>
     </row>
@@ -1588,25 +1576,25 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>52.25</v>
+        <v>52.33</v>
       </c>
       <c r="C11" t="n">
-        <v>55.95</v>
+        <v>56.8</v>
       </c>
       <c r="D11" t="n">
-        <v>60.03</v>
+        <v>60.12</v>
       </c>
       <c r="E11" t="n">
-        <v>60.27</v>
+        <v>60.33</v>
       </c>
       <c r="F11" t="n">
-        <v>64.81</v>
+        <v>64.81999999999999</v>
       </c>
       <c r="G11" t="n">
-        <v>65.08</v>
+        <v>65.59999999999999</v>
       </c>
       <c r="H11" t="n">
-        <v>67.25</v>
+        <v>68</v>
       </c>
       <c r="I11" t="n">
         <v>38</v>
@@ -1615,7 +1603,7 @@
         <v>92</v>
       </c>
       <c r="K11" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="12">
@@ -1625,10 +1613,10 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>43.9</v>
+        <v>44.01</v>
       </c>
       <c r="C12" t="n">
-        <v>46.16</v>
+        <v>47.22</v>
       </c>
       <c r="D12" t="n">
         <v>47.75</v>
@@ -1637,10 +1625,10 @@
         <v>47.75</v>
       </c>
       <c r="F12" t="n">
-        <v>48.58</v>
+        <v>49.16</v>
       </c>
       <c r="G12" t="n">
-        <v>49.18</v>
+        <v>49.29</v>
       </c>
       <c r="H12" t="n">
         <v>50</v>
@@ -1649,10 +1637,10 @@
         <v>36.71</v>
       </c>
       <c r="J12" t="n">
-        <v>55.33</v>
+        <v>56.28</v>
       </c>
       <c r="K12" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="13">
@@ -1767,7 +1755,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-28</t>
         </is>
       </c>
     </row>
@@ -1803,7 +1791,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>1.025 (auto — vs 1.025 auto)</t>
+          <t>1.053 (auto — vs 1.053 auto)</t>
         </is>
       </c>
     </row>
@@ -1815,7 +1803,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>1.025</t>
+          <t>1.053</t>
         </is>
       </c>
     </row>
@@ -2032,12 +2020,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-08 15:10:12</t>
+          <t>2026-09-28 10:25:48</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -2052,12 +2040,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.025</t>
+          <t>1.053</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>1.025</t>
+          <t>1.053</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">

</xml_diff>

<commit_message>
Nueva reserva Eva Hoppmann (HM4YH2FDWZ) + cancelación Heidrun Bley (HMRAT8R2PC)
</commit_message>
<xml_diff>
--- a/output/pricing_output.xlsx
+++ b/output/pricing_output.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X7"/>
+  <dimension ref="A1:X8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -613,10 +613,10 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>41.1</v>
+        <v>45.6</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>52.33</v>
@@ -642,19 +642,19 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>baja antelación (↓10%) + pickup fuerte (↑10%) + hueco muy corto (↓10%)</t>
+          <t>antelación muy baja (↓20%) + pickup fuerte (↑10%) + hueco muy corto (↓10%)</t>
         </is>
       </c>
       <c r="O2" s="2" t="n">
-        <v>54.12</v>
+        <v>53.67</v>
       </c>
       <c r="P2" s="2" t="n">
-        <v>48.71</v>
+        <v>48.3</v>
       </c>
       <c r="Q2" s="2" t="n"/>
       <c r="R2" s="2" t="inlineStr">
         <is>
-          <t>Ocupación (hueco muy corto + baja antelación). Objetivo: convertir rápido, evitar hueco vacío. Ajustes en zona: baja antelación (↓10%) + pickup fuerte (↑10%) + hueco muy corto (↓10%).</t>
+          <t>Ocupación (hueco muy corto + antelación muy baja). Objetivo: convertir rápido, evitar hueco vacío. Ajustes en zona: antelación muy baja (↓20%) + pickup fuerte (↑10%) + hueco muy corto (↓10%).</t>
         </is>
       </c>
       <c r="S2" s="2" t="n"/>
@@ -701,10 +701,10 @@
         </is>
       </c>
       <c r="F3" s="2" t="n">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>34.4</v>
+        <v>38.9</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>52.33</v>
@@ -730,27 +730,23 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>pickup fuerte (↑10%) + hueco muy corto (↓10%)</t>
+          <t>baja antelación (↓10%) + pickup fuerte (↑10%) + hueco muy corto (↓10%)</t>
         </is>
       </c>
       <c r="O3" s="2" t="n">
-        <v>54.56</v>
+        <v>54.12</v>
       </c>
       <c r="P3" s="2" t="n">
-        <v>49.1</v>
+        <v>48.71</v>
       </c>
       <c r="Q3" s="2" t="n"/>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>Ocupación (hueco muy corto + baja ocupación futura). Objetivo: convertir rápido, evitar hueco vacío. Ajustes en zona: pickup fuerte (↑10%) + hueco muy corto (↓10%).</t>
+          <t>Ocupación (hueco muy corto + baja antelación). Objetivo: convertir rápido, evitar hueco vacío. Ajustes en zona: baja antelación (↓10%) + pickup fuerte (↑10%) + hueco muy corto (↓10%).</t>
         </is>
       </c>
       <c r="S3" s="2" t="n"/>
-      <c r="T3" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-04</t>
-        </is>
-      </c>
+      <c r="T3" s="2" t="n"/>
       <c r="U3" s="2" t="inlineStr">
         <is>
           <t>2026-10-12</t>
@@ -758,7 +754,7 @@
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>Revisar 2026-10-04; sin vender → bajar 5–10%</t>
+          <t>Revisar 2026-10-12; sin vender → precio Ocupación</t>
         </is>
       </c>
       <c r="W3" s="2" t="n">
@@ -793,10 +789,10 @@
         </is>
       </c>
       <c r="F4" s="2" t="n">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>30</v>
+        <v>34.4</v>
       </c>
       <c r="H4" s="2" t="n">
         <v>52.33</v>
@@ -822,19 +818,19 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>pickup fuerte (↑10%) + hueco muy corto (↓10%)</t>
+          <t>baja antelación (↓10%) + pickup fuerte (↑10%) + hueco muy corto (↓10%)</t>
         </is>
       </c>
       <c r="O4" s="2" t="n">
-        <v>54.56</v>
+        <v>54.12</v>
       </c>
       <c r="P4" s="2" t="n">
-        <v>49.1</v>
+        <v>48.71</v>
       </c>
       <c r="Q4" s="2" t="n"/>
       <c r="R4" s="2" t="inlineStr">
         <is>
-          <t>Ocupación (hueco muy corto + baja ocupación futura). Objetivo: convertir rápido, evitar hueco vacío. Ajustes en zona: pickup fuerte (↑10%) + hueco muy corto (↓10%).</t>
+          <t>Ocupación (hueco muy corto + baja antelación + baja ocupación futura). Objetivo: convertir rápido, evitar hueco vacío. Ajustes en zona: baja antelación (↓10%) + pickup fuerte (↑10%) + hueco muy corto (↓10%).</t>
         </is>
       </c>
       <c r="S4" s="2" t="n"/>
@@ -885,10 +881,10 @@
         </is>
       </c>
       <c r="F5" s="3" t="n">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>23.3</v>
+        <v>27.8</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>44.01</v>
@@ -918,22 +914,18 @@
         </is>
       </c>
       <c r="O5" s="3" t="n">
-        <v>48.53</v>
+        <v>48.46</v>
       </c>
       <c r="P5" s="3" t="n">
-        <v>43.68</v>
+        <v>43.61</v>
       </c>
       <c r="Q5" s="3" t="n"/>
       <c r="R5" s="3" t="inlineStr">
         <is>
-          <t>Equilibrio (temporada baja + antelación adecuada). Precio de mercado balanceado. Ajustes en zona: pickup fuerte (↑10%) + baja ocupación futura (↓10%).</t>
-        </is>
-      </c>
-      <c r="S5" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-02</t>
-        </is>
-      </c>
+          <t>Equilibrio (temporada baja). Precio de mercado balanceado. Ajustes en zona: pickup fuerte (↑10%) + baja ocupación futura (↓10%).</t>
+        </is>
+      </c>
+      <c r="S5" s="3" t="n"/>
       <c r="T5" s="3" t="inlineStr">
         <is>
           <t>2026-10-17</t>
@@ -946,7 +938,7 @@
       </c>
       <c r="V5" s="3" t="inlineStr">
         <is>
-          <t>Revisar 2026-10-02; sin vender → bajar 5%</t>
+          <t>Revisar 2026-10-17; sin vender → bajar 5–10%</t>
         </is>
       </c>
       <c r="W5" s="3" t="n">
@@ -981,10 +973,10 @@
         </is>
       </c>
       <c r="F6" s="3" t="n">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>23.3</v>
+        <v>27.8</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>44.01</v>
@@ -1055,101 +1047,197 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>2026-12-07</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>2026-12-10</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Diciembre (1-19)</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>baja</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>63</v>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>23.3</v>
+      </c>
+      <c r="H7" s="2" t="n">
+        <v>42.36</v>
+      </c>
+      <c r="I7" s="2" t="n">
+        <v>43.9</v>
+      </c>
+      <c r="J7" s="2" t="n">
+        <v>47.69</v>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>Ocupación</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>P25–P40  (42€–43€)</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="n">
+        <v>42.68</v>
+      </c>
+      <c r="N7" s="2" t="inlineStr">
+        <is>
+          <t>buena antelación (↑15%) + pickup fuerte (↑10%) + hueco corto (↓5%) + baja ocupación futura (↓10%)</t>
+        </is>
+      </c>
+      <c r="O7" s="2" t="n">
+        <v>42.96</v>
+      </c>
+      <c r="P7" s="2" t="n">
+        <v>38.66</v>
+      </c>
+      <c r="Q7" s="2" t="n"/>
+      <c r="R7" s="2" t="inlineStr">
+        <is>
+          <t>Ocupación (hueco corto + temporada baja + baja ocupación futura). Objetivo: convertir rápido, evitar hueco vacío. Ajustes en zona: buena antelación (↑15%) + pickup fuerte (↑10%) + hueco corto (↓5%) + baja ocupación futura (↓10%).</t>
+        </is>
+      </c>
+      <c r="S7" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-07</t>
+        </is>
+      </c>
+      <c r="T7" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-22</t>
+        </is>
+      </c>
+      <c r="U7" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-30</t>
+        </is>
+      </c>
+      <c r="V7" s="2" t="inlineStr">
+        <is>
+          <t>Revisar 2026-11-07; sin vender → bajar 5%</t>
+        </is>
+      </c>
+      <c r="W7" s="2" t="n">
+        <v>42.36</v>
+      </c>
+      <c r="X7" s="2" t="n">
+        <v>53.89</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>2026-12-14</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>2026-12-23</t>
         </is>
       </c>
-      <c r="C7" s="3" t="n">
-        <v>16</v>
-      </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="C8" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
         <is>
           <t>Diciembre (1-19)</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="E8" s="3" t="inlineStr">
         <is>
           <t>baja</t>
         </is>
       </c>
-      <c r="F7" s="3" t="n">
+      <c r="F8" s="3" t="n">
         <v>70</v>
       </c>
-      <c r="G7" s="3" t="n">
+      <c r="G8" s="3" t="n">
         <v>18.9</v>
       </c>
-      <c r="H7" s="3" t="n">
-        <v>42.03</v>
-      </c>
-      <c r="I7" s="3" t="n">
-        <v>43.45</v>
-      </c>
-      <c r="J7" s="3" t="n">
-        <v>46.67</v>
-      </c>
-      <c r="K7" s="3" t="inlineStr">
+      <c r="H8" s="3" t="n">
+        <v>42.36</v>
+      </c>
+      <c r="I8" s="3" t="n">
+        <v>43.9</v>
+      </c>
+      <c r="J8" s="3" t="n">
+        <v>47.69</v>
+      </c>
+      <c r="K8" s="3" t="inlineStr">
         <is>
           <t>Equilibrio</t>
         </is>
       </c>
-      <c r="L7" s="3" t="inlineStr">
-        <is>
-          <t>P45–P60  (43€–45€)</t>
-        </is>
-      </c>
-      <c r="M7" s="3" t="n">
-        <v>43.83</v>
-      </c>
-      <c r="N7" s="3" t="inlineStr">
+      <c r="L8" s="3" t="inlineStr">
+        <is>
+          <t>P45–P60  (43€–46€)</t>
+        </is>
+      </c>
+      <c r="M8" s="3" t="n">
+        <v>44.58</v>
+      </c>
+      <c r="N8" s="3" t="inlineStr">
         <is>
           <t>buena antelación (↑15%) + pickup fuerte (↑10%) + baja ocupación futura (↓10%)</t>
         </is>
       </c>
-      <c r="O7" s="3" t="n">
-        <v>44.07</v>
-      </c>
-      <c r="P7" s="3" t="n">
-        <v>39.66</v>
-      </c>
-      <c r="Q7" s="3" t="n">
-        <v>293.07</v>
-      </c>
-      <c r="R7" s="3" t="inlineStr">
+      <c r="O8" s="3" t="n">
+        <v>44.91</v>
+      </c>
+      <c r="P8" s="3" t="n">
+        <v>40.42</v>
+      </c>
+      <c r="Q8" s="3" t="n">
+        <v>298.65</v>
+      </c>
+      <c r="R8" s="3" t="inlineStr">
         <is>
           <t>Equilibrio (temporada baja + antelación adecuada). Precio de mercado balanceado. Ajustes en zona: buena antelación (↑15%) + pickup fuerte (↑10%) + baja ocupación futura (↓10%).</t>
         </is>
       </c>
-      <c r="S7" s="3" t="inlineStr">
-        <is>
-          <t>2026-11-07</t>
-        </is>
-      </c>
-      <c r="T7" s="3" t="inlineStr">
-        <is>
-          <t>2026-11-22</t>
-        </is>
-      </c>
-      <c r="U7" s="3" t="inlineStr">
-        <is>
-          <t>2026-11-30</t>
-        </is>
-      </c>
-      <c r="V7" s="3" t="inlineStr">
-        <is>
-          <t>Revisar 2026-11-07; sin vender → bajar 5%</t>
-        </is>
-      </c>
-      <c r="W7" s="3" t="n">
-        <v>42.03</v>
-      </c>
-      <c r="X7" s="3" t="n">
-        <v>52.74</v>
+      <c r="S8" s="3" t="inlineStr">
+        <is>
+          <t>2026-11-14</t>
+        </is>
+      </c>
+      <c r="T8" s="3" t="inlineStr">
+        <is>
+          <t>2026-11-29</t>
+        </is>
+      </c>
+      <c r="U8" s="3" t="inlineStr">
+        <is>
+          <t>2026-12-07</t>
+        </is>
+      </c>
+      <c r="V8" s="3" t="inlineStr">
+        <is>
+          <t>Revisar 2026-11-14; sin vender → bajar 5%</t>
+        </is>
+      </c>
+      <c r="W8" s="3" t="n">
+        <v>42.36</v>
+      </c>
+      <c r="X8" s="3" t="n">
+        <v>53.89</v>
       </c>
     </row>
   </sheetData>
@@ -1650,25 +1738,25 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>42.03</v>
+        <v>42.36</v>
       </c>
       <c r="C13" t="n">
         <v>43</v>
       </c>
       <c r="D13" t="n">
-        <v>43.05</v>
+        <v>43.45</v>
       </c>
       <c r="E13" t="n">
-        <v>43.45</v>
+        <v>43.9</v>
       </c>
       <c r="F13" t="n">
-        <v>44.62</v>
+        <v>45.7</v>
       </c>
       <c r="G13" t="n">
-        <v>45.43</v>
+        <v>46.35</v>
       </c>
       <c r="H13" t="n">
-        <v>46.67</v>
+        <v>47.69</v>
       </c>
       <c r="I13" t="n">
         <v>38.33</v>
@@ -1677,7 +1765,7 @@
         <v>51.5</v>
       </c>
       <c r="K13" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="14">
@@ -1755,7 +1843,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-05</t>
         </is>
       </c>
     </row>
@@ -1791,7 +1879,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>1.053 (auto — vs 1.053 auto)</t>
+          <t>1.063 (auto — vs 1.063 auto)</t>
         </is>
       </c>
     </row>
@@ -1803,7 +1891,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>1.053</t>
+          <t>1.063</t>
         </is>
       </c>
     </row>
@@ -2020,12 +2108,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-28 10:25:48</t>
+          <t>2026-10-05 12:17:39</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -2040,17 +2128,17 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.053</t>
+          <t>1.063</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>1.053</t>
+          <t>1.063</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">

</xml_diff>